<commit_message>
Actionnariat : règle fondée sur le contrôle, 4 catégories
- public, groupe étranger, mixte, privé sans contrôle étranger
  (spécification 5.3, tableau des preuves).
- BH public : État + entreprises publiques 55,63 % (rapport annuel 2025).
- BTE mixte ; Attijari : contrôle d'Attijariwafa bank écrit dans la
  plaquette financière d'avril 2022.
- banques.xlsx, README et PDF de docs/ mis à jour.
</commit_message>
<xml_diff>
--- a/donnees_reference/banques.xlsx
+++ b/donnees_reference/banques.xlsx
@@ -552,7 +552,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>privé tunisien</t>
+          <t>privé sans contrôle étranger</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
@@ -677,7 +677,7 @@
       <c r="K4" s="5" t="n"/>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t>Groupe Mzabi 9,94 %, groupe Driss 9,54 %. 2019 : Attijariwafa bank (Maroc) s'engage à maintenir au moins 55 % du capital (TJARI_EF_2019-12.pdf p. 14). À confirmer : le lien Andalu Carthage Holding – Attijariwafa bank n'est écrit dans aucun document lu (déduit : seul actionnaire au-dessus de 55 %).</t>
+          <t>Groupe Mzabi 9,94 %, groupe Driss 9,54 %. Plaquette financière Attijari bank d'avril 2022, p. 1 (attijaribank.com.tn) : « à travers la participation de la société Andalucarthage Holding, le Groupe Attijariwafa bank est l'actionnaire de référence qui détient la majorité des droits de vote et assure le contrôle de l'institution » (58,98 % au 31/12/2021). 2019 : Attijariwafa bank s'engage à maintenir au moins 55 % du capital (TJARI_EF_2019-12.pdf p. 14).</t>
         </is>
       </c>
     </row>
@@ -700,30 +700,34 @@
       <c r="D5" s="4" t="n">
         <v>33.37</v>
       </c>
-      <c r="E5" s="2" t="n"/>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
           <t>État tunisien</t>
         </is>
       </c>
       <c r="G5" s="5" t="n">
-        <v>46142</v>
+        <v>46022</v>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>Bourse de Tunis, fiche émetteur (AGO du 30/04/2026) : https://www.tunis-stockexchange.com/informations-bh-bank</t>
+          <t>Rapport annuel BH Bank 2025 (rapport à l'AGO, bhbank.tn, RAPPORT-2025-AGO-BHBANK.pdf)</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>rubrique 4 « Principaux actionnaires »</t>
+          <t>19 (page 21 du PDF)</t>
         </is>
       </c>
       <c r="J5" s="5" t="n"/>
       <c r="K5" s="5" t="n"/>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>ETAP 16,57 %, groupe Horchani 23,19 %, actionnaires de moins de 5 % 26,87 % (non détaillés). État + ETAP = 49,94 % : la règle des 50 % ne peut pas être appliquée sans le détail des petits actionnaires publics. BH_EF_2025-12_cmf.pdf p. 48 : « l'État tunisien (principal actionnaire) ». Actionnariat de 2019 non trouvé (bhbank.tn : rapport 2025 seulement, tableau d'actionnariat sans texte).</t>
+          <t>Tableau « Actionnariat » : État tunisien 33,37 %, entreprises publiques 22,26 % (dont ETAP 16,57 %), entreprises parapubliques 1,02 %, personnes morales privées 28,70 %, personnes physiques 14,50 %, étrangers 0,10 %. État + entreprises publiques = 55,63 % : contrôle public. Fiche Bourse (AGO du 30/04/2026) : État 33,37 %, ETAP 16,57 %, groupe Horchani 23,19 %. BH_EF_2025-12_cmf.pdf p. 48 : « l'État tunisien (principal actionnaire) ». Actionnariat de 2019 non trouvé (bhbank.tn : rapport 2025 seulement).</t>
         </is>
       </c>
     </row>
@@ -748,7 +752,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>privé tunisien</t>
+          <t>privé sans contrôle étranger</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -848,7 +852,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>privé tunisien</t>
+          <t>privé sans contrôle étranger</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -873,7 +877,7 @@
       <c r="K8" s="5" t="n"/>
       <c r="L8" s="3" t="inlineStr">
         <is>
-          <t>Groupe El Fekih 10 %, groupe Kammoun 9,52 %, autres 45,15 %. BFCM = « entité exerçant une influence notable sur la BT » (BT_EF_2019-12.pdf p. 65), pas un actionnaire de contrôle : privé tunisien par la règle. À confirmer.</t>
+          <t>Groupe El Fekih 10 %, groupe Kammoun 9,52 %, autres 45,15 %. BFCM = « entité exerçant une influence notable sur la BT » (BT_EF_2019-12.pdf p. 65), pas un actionnaire de contrôle : privé sans contrôle étranger.</t>
         </is>
       </c>
     </row>
@@ -896,8 +900,16 @@
       <c r="D9" s="4" t="n">
         <v>38.9</v>
       </c>
-      <c r="E9" s="2" t="n"/>
-      <c r="F9" s="3" t="n"/>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>mixte</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>État tunisien / ADIA</t>
+        </is>
+      </c>
       <c r="G9" s="5" t="n">
         <v>43830</v>
       </c>
@@ -917,7 +929,7 @@
       </c>
       <c r="L9" s="3" t="inlineStr">
         <is>
-          <t>Chacun 38,9 % du capital et 50 % des droits de vote ; ADP 22,2 % sans droit de vote. Inchangé au 30/06/2024 (BTE_EF_2024-06.pdf p. 24). Contrôle conjoint : la règle ne tranche pas (public 38,9 % &lt; 50 %, ADIA sans contrôle seul).</t>
+          <t>Chacun 38,9 % du capital et 50 % des droits de vote ; ADP 22,2 % sans droit de vote. Inchangé au 30/06/2024 (BTE_EF_2024-06.pdf p. 24). Contrôle conjoint public / étranger : mixte.</t>
         </is>
       </c>
     </row>
@@ -940,8 +952,16 @@
       <c r="D10" s="4" t="n">
         <v>40.8</v>
       </c>
-      <c r="E10" s="2" t="n"/>
-      <c r="F10" s="3" t="n"/>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>mixte</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>État tunisien / ADIA</t>
+        </is>
+      </c>
       <c r="G10" s="5" t="n">
         <v>45657</v>
       </c>
@@ -961,7 +981,7 @@
       <c r="K10" s="5" t="n"/>
       <c r="L10" s="3" t="inlineStr">
         <is>
-          <t>Augmentation de capital (AGE prévue le 30/04/2024, BTE_EF_2023-12.pdf p. 42), faite entre le 30/06/2024 et le 31/12/2024 (date exacte non trouvée). État 32,19 % (39 % des droits de vote), La Poste tunisienne 8,62 % (11 %), ADIA 40,80 % (50 %), ADP 18,39 %. Même structure à la fiche Bourse (AGO du 30/04/2026). Public : 40,81 % du capital, 50 % des droits de vote : la règle ne tranche pas.</t>
+          <t>Augmentation de capital (AGE prévue le 30/04/2024, BTE_EF_2023-12.pdf p. 42), faite entre le 30/06/2024 et le 31/12/2024 (date exacte non trouvée). État 32,19 % (39 % des droits de vote), La Poste tunisienne 8,62 % (11 %), ADIA 40,80 % (50 %), ADP 18,39 %. Même structure à la fiche Bourse (AGO du 30/04/2026). Droits de vote : 50 % public (État + La Poste), 50 % ADIA : contrôle conjoint, mixte.</t>
         </is>
       </c>
     </row>
@@ -1088,7 +1108,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>privé tunisien</t>
+          <t>privé sans contrôle étranger</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
@@ -1190,7 +1210,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>privé tunisien</t>
+          <t>privé sans contrôle étranger</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
@@ -1217,7 +1237,7 @@
       </c>
       <c r="L15" s="3" t="inlineStr">
         <is>
-          <t>2019 : ICD 30 %, groupe STB 17,16 %, M. Mohamed Hédi Ben Ayed 11,93 %, CDC 10 %, MM. Hamrouni 6,61 % et 6,19 %, Medimix 5 %. 31/12/2021 : ICD 30 %, groupe Ben Ayed 22,82 %, groupe STB 18,43 %, CDC 10 % (rapport annuel 2021, p. 13). Public (groupe STB + CDC) 27 à 28 % ; ICD, premier actionnaire sans majorité, n'est pas actionnaire de contrôle : privé tunisien par la règle. À confirmer.</t>
+          <t>2019 : ICD 30 %, groupe STB 17,16 %, M. Mohamed Hédi Ben Ayed 11,93 %, CDC 10 %, MM. Hamrouni 6,61 % et 6,19 %, Medimix 5 %. 31/12/2021 : ICD 30 %, groupe Ben Ayed 22,82 %, groupe STB 18,43 %, CDC 10 % (rapport annuel 2021, p. 13). Public (groupe STB + CDC) 27 à 28 % ; ICD, premier actionnaire sans majorité, n'est pas actionnaire de contrôle : privé sans contrôle étranger.</t>
         </is>
       </c>
     </row>
@@ -1242,7 +1262,7 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>privé tunisien</t>
+          <t>privé sans contrôle étranger</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Actionnariat BTE sans trou, ouverture du projet par un tiers
- BTE : date de l'augmentation de capital de 2024 introuvable dans les états
  financiers ; seconde période d'actionnariat au 01/07/2024 (date exacte
  inconnue, entre le 30/06 et le 31/12/2024), avec la source de la décision et
  l'indice des capitaux propres trimestriels.
- tests/test_actionnariat.py : périodes continues de 2019 à aujourd'hui pour les
  12 banques, catégories et sources (41 tests).
- Cache des données Power BI retiré du .gitignore (données publiques), pour
  ouvrir le projet sans réglage ; il sera versionné après une vérification.
- README : section « Ouvrir le rapport » ; publication sur le web prévue à la fin.
- Spécification 5.3, guide, feuille de route, PDF ; TMDL réenregistré par Power BI.
</commit_message>
<xml_diff>
--- a/donnees_reference/banques.xlsx
+++ b/donnees_reference/banques.xlsx
@@ -976,12 +976,12 @@
         </is>
       </c>
       <c r="J10" s="5" t="n">
-        <v>45657</v>
+        <v>45474</v>
       </c>
       <c r="K10" s="5" t="n"/>
       <c r="L10" s="3" t="inlineStr">
         <is>
-          <t>Augmentation de capital (AGE prévue le 30/04/2024, BTE_EF_2023-12.pdf p. 42), faite entre le 30/06/2024 et le 31/12/2024 (date exacte non trouvée). État 32,19 % (39 % des droits de vote), La Poste tunisienne 8,62 % (11 %), ADIA 40,80 % (50 %), ADP 18,39 %. Même structure à la fiche Bourse (AGO du 30/04/2026). Droits de vote : 50 % public (État + La Poste), 50 % ADIA : contrôle conjoint, mixte.</t>
+          <t>Augmentation de capital (AGE prévue le 30/04/2024, BTE_EF_2023-12.pdf p. 42 ; décidée par l'AGE du 30/04/2024, BTE_EF_2024-06.pdf p. 32) : date exacte inconnue, entre le 30/06 et le 31/12/2024 (capital 90 000 → 108 744 kDT, BTE_EF_2024-12.pdf p. 31 ; aucune date dans les notes de 2024 et 2025) ; début de période fixé au 01/07/2024 pour que les périodes se suivent. Indice non confirmé : capitaux propres trimestriels 41,704 MDT au 30/06/2024 (BTE_2025T2.pdf p. 1) et 62,764 MDT au 30/09/2024 (BTE_2025T3.pdf p. 1). État 32,19 % (39 % des droits de vote), La Poste tunisienne 8,62 % (11 %), ADIA 40,80 % (50 %), ADP 18,39 %. Même structure à la fiche Bourse (AGO du 30/04/2026). Droits de vote : 50 % public (État + La Poste), 50 % ADIA : contrôle conjoint, mixte.</t>
         </is>
       </c>
     </row>

</xml_diff>